<commit_message>
RIO-DSL-UPDATE: Documentacion.xlsx al dia (cambios 2026-10-12 a 10-14) y pendiente de campo del salto de MODO 2
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Documentación.xlsx
+++ b/Documentación.xlsx
@@ -780,7 +780,7 @@
       </c>
       <c r="G5" s="4" t="inlineStr">
         <is>
-          <t>Rampa de llenado hasta PRESION_OBJETIVO_LOCAL en TIEMPO_LLENADO_S</t>
+          <t>Rampa del objetivo desde la presión al entrar hasta PRESION_OBJETIVO_LOCAL en TIEMPO_LLENADO_S, nunca más rápido que 0.35 PSI/s (0 = al tope). Si llega con el objetivo aplicado más arriba (volviendo de MODO 2 o de CALIB 12) baja a objetivo/T, o 0.35 PSI/s con T=0 (2026-10-14)</t>
         </is>
       </c>
     </row>
@@ -812,7 +812,7 @@
       </c>
       <c r="F6" s="25" t="inlineStr">
         <is>
-          <t>Solo desde MODO 1 (o ya en MODO 2). Requiere PRESION_OBJETIVO_REMOTO &gt; 0. Rechaza los demás. Además exige enlace LoRa y aspersor reportando (2026-10-02)</t>
+          <t>Solo desde MODO 1 (o ya en MODO 2) y con el llenado de MODO 1 TERMINADO: rampa ya en PRESION_OBJETIVO_LOCAL y presión a &lt;= 2 PSI (2026-10-14). Requiere PRESION_OBJETIVO_REMOTO &gt; 0. Rechaza los demás. Además exige enlace LoRa y aspersor reportando (2026-10-02). La vuelta automática 1→2 tras una degradación no pide el llenado</t>
         </is>
       </c>
       <c r="G6" s="4" t="inlineStr">
@@ -978,14 +978,14 @@
     <row r="14" ht="62.1" customHeight="1" s="23">
       <c r="C14" s="14" t="inlineStr">
         <is>
-          <t>NOTA 3 [IMPLEMENTADA 2026-10-01] - Un downlink/comando MODO rechazado (motor detenido, objetivo remoto sin configurar, MODO 2 sin venir de MODO 1) responde con el ACK del downlink (FPort 3: ID, STATUS, VALOR) y además fuerza un uplink inmediato con la alerta 13 "modo rechazado" (transitoria: después se restaura la alerta anterior). Pendiente: sumar la alerta 13 al decoder de AWS.</t>
+          <t>NOTA 3 [IMPLEMENTADA 2026-10-01] - Un downlink/comando MODO rechazado (motor detenido, objetivo remoto sin configurar, MODO 2 sin venir de MODO 1, MODO 2 con el llenado de MODO 1 sin terminar) responde con el ACK del downlink (FPort 3: ID, STATUS, VALOR) y además fuerza un uplink inmediato con la alerta 13 "modo rechazado" (transitoria: después se restaura la alerta anterior). Pendiente: sumar la alerta 13 al decoder de AWS.</t>
         </is>
       </c>
     </row>
     <row r="15" ht="62.1" customHeight="1" s="23">
       <c r="C15" s="14" t="inlineStr">
         <is>
-          <t>NOTA 4 - MODO 1 se acepta desde cualquier MODO con motor encendido (decisión 2026-10-01: no se agregan restricciones). La única restricción de entrada es la de MODO 2: solo desde MODO 1. Las reglas viven en modo_fsm.c (Modo_ValidarEntrada).</t>
+          <t>NOTA 4 - MODO 1 se acepta desde cualquier MODO con motor encendido (decisión 2026-10-01: no se agregan restricciones). La única restricción de entrada es la de MODO 2: solo desde MODO 1 y con el llenado terminado (2026-10-14). Las reglas viven en modo_fsm.c (Modo_ValidarEntrada). Al entrar a MODO 1 con el motor acelerado (más de 30 RPM sobre RPM_MIN, ej. degradación 3→1) el PID#2 arranca desde la RPM real</t>
         </is>
       </c>
     </row>
@@ -1368,7 +1368,7 @@
       </c>
       <c r="F7" s="24" t="inlineStr">
         <is>
-          <t>MODO 0 (solo si SET_PRESION está activo; con SET_RPM no se usa el sensor)</t>
+          <t>MODO 0. En MODO 3 con SET_RPM (2026-10-14): si el sensor pasa de válido a inválido, ralentí + SET_RPM = 0 y MODO 0 a los 60 s; si ya estaba inválido desde antes (banco sin sensor) no hace nada</t>
         </is>
       </c>
       <c r="G7" s="24" t="inlineStr">
@@ -1516,7 +1516,7 @@
       </c>
       <c r="B11" s="24" t="inlineStr">
         <is>
-          <t>Motor detenido pidiendo MODO 1/2, MODO 2 sin PRESION_OBJETIVO_REMOTO, o MODO 2 sin venir de MODO 1</t>
+          <t>Motor detenido pidiendo MODO 1/2, MODO 2 sin PRESION_OBJETIVO_REMOTO, o MODO 2 sin venir de MODO 1, o MODO 2 con el llenado de MODO 1 sin terminar (2026-10-14)</t>
         </is>
       </c>
       <c r="C11" s="24" t="inlineStr">
@@ -1681,7 +1681,7 @@
     <row r="1">
       <c r="A1" s="22" t="inlineStr">
         <is>
-          <t>PRUEBAS Y CALIBRACIONES (parámetro CALIB), según el código al 2026-10-01. Todas SOLO en MODO 4 (excepto CALIB 12, que también arranca desde MODO 1)</t>
+          <t>PRUEBAS Y CALIBRACIONES (parámetro CALIB), según el código al 2026-10-14. Todas SOLO en MODO 4 (excepto CALIB 12, que también arranca desde MODO 1)</t>
         </is>
       </c>
     </row>
@@ -2198,12 +2198,12 @@
       </c>
       <c r="C12" s="24" t="inlineStr">
         <is>
-          <t>MODO 4, CALIB previo 0, motor operando CON la bomba embragada, PRESION_OBJETIVO_LOCAL y TIEMPO_LLENADO_S configurados, PRESION_MAX &gt; objetivo</t>
+          <t>MODO 4, CALIB previo 0, motor operando CON la bomba embragada, PRESION_OBJETIVO_LOCAL configurado (TIEMPO_LLENADO_S = 0 usa 300 s), PRESION_MAX &gt; objetivo</t>
         </is>
       </c>
       <c r="D12" s="24" t="inlineStr">
         <is>
-          <t>ESPERA → BASE (5 s) → SUBIDA al ritmo de TIEMPO_LLENADO_S; calcula la K por tramos</t>
+          <t>ESPERA → BASE (5 s) → SUBIDA al ritmo de TIEMPO_LLENADO_S, nunca más rápido que 0.35 PSI/s; calcula la K por tramos</t>
         </is>
       </c>
       <c r="E12" s="24" t="inlineStr">
@@ -2353,7 +2353,7 @@
       </c>
       <c r="D15" s="24" t="inlineStr">
         <is>
-          <t>ESPERA, LLENADO (solo desde MODO 4), BASE, ESCALÓN (±5 PSI), VOLVER, VALIDAR, FINALIZANDO</t>
+          <t>ESPERA, LLENADO (solo desde MODO 4), BASE, ESCALÓN (±5 PSI), VOLVER, VALIDAR. Aborta si el aspersor no es creíble en la base (0 o &lt; 20 % de la presión local), si no responde al escalón (4 reportes sin moverse 1.5 PSI con la local ya llegada) o si se mueve al revés más de 3 PSI (2026-10-14). Desde MODO 1, al terminar o abortar la rampa de MODO 1 regresa el objetivo a la base (ya no hay estado FINALIZANDO)</t>
         </is>
       </c>
       <c r="E15" s="24" t="inlineStr">
@@ -2448,7 +2448,7 @@
       </c>
       <c r="C17" s="24" t="inlineStr">
         <is>
-          <t>MODO 4, CALIB previo 0, motor operando CON la bomba embragada, PID_RPM_KP &gt; 0, PRESION_OBJETIVO_LOCAL y TIEMPO_LLENADO_S configurados</t>
+          <t>MODO 4, CALIB previo 0, motor operando CON la bomba embragada, PID_RPM_KP &gt; 0, PRESION_OBJETIVO_LOCAL configurado (TIEMPO_LLENADO_S = 0 usa 300 s)</t>
         </is>
       </c>
       <c r="D17" s="24" t="inlineStr">
@@ -2813,7 +2813,7 @@
       </c>
       <c r="D12" s="24" t="inlineStr">
         <is>
-          <t>Se reinicia solo en el flanco de entrada (MODO 1↔2 no reinicia) y al terminar el retroceso de MODO 2</t>
+          <t>Se reinicia en el flanco de entrada (MODO 1↔2 no reinicia), al terminar el retroceso de MODO 2 y al volver el sensor de una falla (2026-10-14). Arranca desde la RPM real (bumpless) en MODO 3 y en MODO 1 si el motor viene a más de RPM_MIN + 30</t>
         </is>
       </c>
       <c r="E12" s="24" t="inlineStr">
@@ -2845,7 +2845,7 @@
       </c>
       <c r="E13" s="24" t="inlineStr">
         <is>
-          <t>Objetivo local aplicado &lt;= PRESION_MAX × 0.95</t>
+          <t>Objetivo local aplicado &lt;= PRESION_MAX (100 %, desde 2026-10-12; era × 0.95)</t>
         </is>
       </c>
     </row>
@@ -2862,17 +2862,17 @@
       </c>
       <c r="C14" s="24" t="inlineStr">
         <is>
-          <t>Objetivo sube a la velocidad de llenado (PRESION_OBJETIVO_LOCAL / TIEMPO_LLENADO_S) desde la presión medida al entrar; solo hacia arriba</t>
+          <t>Objetivo aplicado que avanza cada vuelta: sube a (objetivo − presión al entrar) / TIEMPO_LLENADO_S, nunca más rápido que 0.35 PSI/s (T = 0 → al tope); baja a objetivo / T (o 0.35 PSI/s) cuando viene de MODO 2 o de CALIB 12</t>
         </is>
       </c>
       <c r="D14" s="24" t="inlineStr">
         <is>
-          <t>Se omite en MODO 3, MODO 2 y CALIB 10/11/14</t>
+          <t>Se omite en MODO 3 (su propio tope de 0.35 PSI/s), MODO 2, CALIB 12 y CALIB 9/10/11/14; mientras tanto copia el objetivo que ellos aplican, así al volver a MODO 1 no salta (2026-10-14)</t>
         </is>
       </c>
       <c r="E14" s="24" t="inlineStr">
         <is>
-          <t>Con tasa 0 va directo al objetivo</t>
+          <t>Con el sensor en falla se re-ancla en la presión medida</t>
         </is>
       </c>
     </row>
@@ -2889,7 +2889,7 @@
       </c>
       <c r="C15" s="24" t="inlineStr">
         <is>
-          <t>Objetivo local aplicado cambia a la velocidad de llenado (PRESION_OBJETIVO_LOCAL / TIEMPO_LLENADO_S) en ambos sentidos</t>
+          <t>Objetivo local aplicado: sube como máximo a 0.35 PSI/s (desde 2026-10-13) y baja a la velocidad de llenado (PRESION_OBJETIVO_LOCAL / TIEMPO_LLENADO_S; con 0, directo). Con el sensor en falla se re-ancla en la presión medida (2026-10-14)</t>
         </is>
       </c>
       <c r="D15" s="24" t="n"/>
@@ -2903,22 +2903,22 @@
       </c>
       <c r="B16" s="24" t="inlineStr">
         <is>
-          <t>Presión &gt; PRESION_MAX</t>
+          <t>Presión &gt; PRESION_MAX 1 s seguido (filtrada o rápida)</t>
         </is>
       </c>
       <c r="C16" s="24" t="inlineStr">
         <is>
-          <t>Con carga inferida (MODO 1/2/3 y MODO 4 durante las pruebas de presión). El detalle exacto cambió el 2026-10-01: revisar contra main.c</t>
+          <t>Se dispara solo con carga inferida (MODO 1/2/3 y MODO 4 durante CALIB 9/10/11/12/14). La lectura rápida es el promedio de 0.5 s sin el limitador de 0.4 PSI/s. PRESION_MAX acepta como máximo 150 (fondo de escala del sensor)</t>
         </is>
       </c>
       <c r="D16" s="24" t="inlineStr">
         <is>
-          <t>setpoint = 0 y servo cae a MIN; alerta 5; se libera a &lt;= 0.9 × PRESION_MAX</t>
+          <t>setpoint = 0 y servo cae a MIN; alerta 5; aborta CALIB 9/12/14; en MODO 3 borra SET_RPM/SET_PRESION. Se libera cuando las dos lecturas bajan a &lt;= 0.9 × PRESION_MAX y vuelve la alerta anterior</t>
         </is>
       </c>
       <c r="E16" s="24" t="inlineStr">
         <is>
-          <t>No cambia MODO. No actúa sobre CALIB 4, 5 ni la curva del 13</t>
+          <t>No cambia MODO. Con el sensor inválido no se suelta; el estado sigue a la presión aunque se pase a MODO 0 (2026-10-14)</t>
         </is>
       </c>
     </row>
@@ -2989,12 +2989,12 @@
       </c>
       <c r="C19" s="24" t="inlineStr">
         <is>
-          <t>En cada reporte del aspersor: saturado y remota &lt; objetivo × 0.95. Cuenta intentos</t>
+          <t>En cada reporte del aspersor: saturado (RPM_MAX_CARGA o techo local) y remota &lt; objetivo × 0.95. Cuenta intentos; el contador vuelve a 0 solo cuando el aspersor llega a su banda (2026-10-14; antes se borraba en el primer reporte no saturado y nunca llegaba al 4º)</t>
         </is>
       </c>
       <c r="D19" s="24" t="inlineStr">
         <is>
-          <t>Intentos 1-3: retroceso de 20 s con setpoint 0. Intento 4: alerta 2 + MODO 0</t>
+          <t>Intentos 1-3: retroceso de 20 s con setpoint 0 + alerta 14. Intento 4: alerta 2 + MODO 0</t>
         </is>
       </c>
       <c r="E19" s="24" t="inlineStr">
@@ -3730,7 +3730,7 @@
       </c>
       <c r="C5" s="24" t="inlineStr">
         <is>
-          <t>Supervisor MODO 2 (fuga): 4º intento. Además MODO=0</t>
+          <t>Supervisor MODO 2 (fuga): 4º intento (el contador solo vuelve a 0 si el aspersor llega a su objetivo). Además MODO=0</t>
         </is>
       </c>
       <c r="D5" s="24" t="inlineStr">
@@ -3750,7 +3750,7 @@
       </c>
       <c r="C6" s="24" t="inlineStr">
         <is>
-          <t>Sensor fuera de 0.2-3.0 V en un modo con cascada local. Tras 60 s seguidos y MODO != 4: MODO 0</t>
+          <t>Sensor fuera de 0.2-3.0 V en un modo con cascada local. Tras 60 s seguidos y MODO != 4: MODO 0. También en MODO 3 con SET_RPM si el sensor se cae estando en MODO 3 (2026-10-14)</t>
         </is>
       </c>
       <c r="D6" s="24" t="inlineStr">
@@ -3790,12 +3790,12 @@
       </c>
       <c r="C8" s="24" t="inlineStr">
         <is>
-          <t>Presión &gt; PRESION_MAX con carga inferida</t>
+          <t>Presión filtrada o rápida &gt; PRESION_MAX durante 1 s, con carga inferida (2026-10-14: la filtrada también pide 1 s)</t>
         </is>
       </c>
       <c r="D8" s="24" t="inlineStr">
         <is>
-          <t>Presión &lt;= 0.9 × PRESION_MAX</t>
+          <t>Las dos lecturas &lt;= 0.9 × PRESION_MAX (con el sensor inválido no se suelta). Vuelve la alerta que había antes</t>
         </is>
       </c>
     </row>
@@ -3935,7 +3935,7 @@
       </c>
       <c r="D15" s="24" t="inlineStr">
         <is>
-          <t>Enlace bueno de nuevo, si el código sigue en 12. Pendiente: sumar a NOMBRES_ALERTA del decoder AWS</t>
+          <t>Enlace bueno de nuevo, si el código sigue en 12</t>
         </is>
       </c>
     </row>
@@ -3955,11 +3955,32 @@
       </c>
       <c r="D16" s="24" t="inlineStr">
         <is>
-          <t>Después de enviar el uplink inmediato que la lleva se restaura la alerta que había. Pendiente: sumar a NOMBRES_ALERTA del decoder AWS</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="45" customHeight="1" s="23"/>
+          <t>Después de enviar el uplink inmediato que la lleva se restaura la alerta que había</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="55" customHeight="1" s="23">
+      <c r="A17" s="24" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="B17" s="24" t="inlineStr">
+        <is>
+          <t>MODO_REMOTO_RETROCESO</t>
+        </is>
+      </c>
+      <c r="C17" s="24" t="inlineStr">
+        <is>
+          <t>Supervisor MODO 2 (fuga): cada retroceso de 20 s a ralentí antes de reintentar (intentos 1-3). Nueva 2026-10-14, ya en decoder.py</t>
+        </is>
+      </c>
+      <c r="D17" s="24" t="inlineStr">
+        <is>
+          <t>Cuando el aspersor llega a su objetivo; el 4º fallo pasa a la alerta 2</t>
+        </is>
+      </c>
+    </row>
     <row r="18">
       <c r="A18" s="24" t="inlineStr">
         <is>
@@ -3968,9 +3989,8 @@
       </c>
     </row>
   </sheetData>
-  <mergeCells count="2">
+  <mergeCells count="1">
     <mergeCell ref="A1:D1"/>
-    <mergeCell ref="A17:D17"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -4229,7 +4249,7 @@
       </c>
       <c r="C13" s="24" t="inlineStr">
         <is>
-          <t>Configuración (RPM_MAX, RPM_MIN, RPM_MAX_CARGA, PRESION_MAX, SERVO_PULSO_*, INTERVALO_*, e IDs desconocidos): rechazada con motor operando</t>
+          <t>Configuración (RPM_MAX, RPM_MIN, RPM_MAX_CARGA, SERVO_PULSO_*, INTERVALO_*, e IDs desconocidos): rechazada con motor operando. PRESION_MAX pasó a proceso el 2026-10-13 (se acepta con el motor encendido, pero en MODO 4)</t>
         </is>
       </c>
       <c r="D13" s="24" t="inlineStr">
@@ -4251,7 +4271,7 @@
       </c>
       <c r="C14" s="24" t="inlineStr">
         <is>
-          <t>SET_RATIO, SET_RATIO_AUTO, RPM_MAX, RPM_MIN, RPM_MAX_CARGA, PRESION_MAX. Ganancias PID_*: MODO 4 con CALIB 0. SERVO_PULSO_MIN/MAX: CALIB 1 o 2</t>
+          <t>SET_RATIO, SET_RATIO_AUTO, RPM_MAX, RPM_MIN, RPM_MAX_CARGA, PRESION_MAX, PRESION_OBJETIVO_LOCAL (2026-10-12), TIEMPO_LLENADO_S (2026-10-14). Ganancias PID_*: MODO 4 con CALIB 0. SERVO_PULSO_MIN/MAX: CALIB 1 o 2</t>
         </is>
       </c>
       <c r="D14" s="24" t="n"/>
@@ -4332,7 +4352,7 @@
       </c>
       <c r="D18" s="24" t="inlineStr">
         <is>
-          <t>El EMA y el limitador de 5 PSI/s están apagados (PRESIONV_FILTROS_ACTIVOS=0)</t>
+          <t>Filtros activos desde 2026-10-07 (EMA 0.08 + limitador 5 PSI/s → la filtrada cambia como máximo 0.4 PSI/s). La guarda PRESION_MAX usa además la lectura rápida (0.5 s, sin filtros)</t>
         </is>
       </c>
     </row>
@@ -4922,7 +4942,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A2:G55"/>
+  <dimension ref="A1:G55"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
   <cols>
     <col width="12.42578125" bestFit="1" customWidth="1" style="23" min="1" max="1"/>
@@ -4935,6 +4955,7 @@
     <col width="13.140625" customWidth="1" style="23" min="8" max="8"/>
   </cols>
   <sheetData>
+    <row r="1"/>
     <row r="2">
       <c r="B2" s="22" t="inlineStr">
         <is>
@@ -5185,6 +5206,9 @@
         </is>
       </c>
     </row>
+    <row r="18"/>
+    <row r="19"/>
+    <row r="20"/>
     <row r="21">
       <c r="B21" s="22" t="inlineStr">
         <is>
@@ -5256,7 +5280,7 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Setear PRESION_OBJETIVO_LOCAL, PRESION_MAX, RPM_MAX, RPM_MIN, RPM_MAX_CARGA y TIEMPO_LLENADO_S (ID 8, segundos de 0 PSI al objetivo; 0 = sin rampa). *RPM_MAX es propio de cada modelo de motor. PRESION_MAX debe ser mayor que el objetivo. El orden ya no importa: la velocidad de llenado se calcula al usarla (objetivo / segundos)</t>
+          <t>Setear PRESION_OBJETIVO_LOCAL, PRESION_MAX, RPM_MAX, RPM_MIN, RPM_MAX_CARGA y TIEMPO_LLENADO_S (ID 8; en MODO 1 = segundos desde la presión al entrar hasta el objetivo, nunca más rápido que 0.35 PSI/s, 0 = al tope; solo en MODO 4). *RPM_MAX es propio de cada modelo de motor. PRESION_MAX debe ser mayor que el objetivo. El orden ya no importa: la velocidad de llenado se calcula al usarla (objetivo / segundos)</t>
         </is>
       </c>
       <c r="D24" s="25" t="inlineStr">
@@ -5570,7 +5594,7 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Setear CALIB 14 (autotune PID#2 completo). Requiere PID_RPM_KP &gt; 0, PRESION_OBJETIVO_LOCAL y TIEMPO_LLENADO_S. Guarda PID_PSI_KP/KI solo si valida. Esperar alerta 8 (OK) o 9 (FALLO). SIN PROBAR con motobomba real</t>
+          <t>Setear CALIB 14 (autotune PID#2 completo). Requiere PID_RPM_KP &gt; 0, PRESION_OBJETIVO_LOCAL y TIEMPO_LLENADO_S. Guarda PID_PSI_KP/KI solo si valida. Esperar alerta 8 (OK) o 9 (FALLO). Probado en campo 2026-10-09 (con tau_c = 2L dio 8.27/1.28, muy rápido; desde 2026-10-12 usa 8L, sin probar)</t>
         </is>
       </c>
       <c r="D40" s="25" t="n"/>
@@ -5613,7 +5637,7 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Solo si se usará MODO 2 (aspersor remoto): setear PRESION_OBJETIVO_REMOTO y correr CALIB 12 (autotune PID#3) desde MODO 4 o desde MODO 1 ya operando. Esperar alerta 10 (OK) u 11 (FALLO). SIN PROBAR</t>
+          <t>Solo si se usará MODO 2 (aspersor remoto): setear PRESION_OBJETIVO_REMOTO y correr CALIB 12 (autotune PID#3) desde MODO 4 o desde MODO 1 ya operando. Esperar alerta 10 (OK) u 11 (FALLO). Probado en campo 2026-10-09 (guardó Ki = 0.01198). Ya no necesita PRESION_OBJETIVO_REMOTO para el ensayo</t>
         </is>
       </c>
       <c r="D42" s="25" t="n"/>

</xml_diff>